<commit_message>
Final Commit with code comments included and notebooks cleaned up
</commit_message>
<xml_diff>
--- a/data/visualizations_public.xlsx
+++ b/data/visualizations_public.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lelandmurrin/Data_Science/Capstone_Project_Accounting_Public/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A805C32B-D871-B047-8066-01A4CE9009BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFD70694-A088-4342-9C85-0D39513892A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1860" windowWidth="29400" windowHeight="17260" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3340" yWindow="740" windowWidth="29400" windowHeight="16960" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lag_stats_CB_172" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="165">
   <si>
     <t>Desc1 CB Comparison Table for Periods 4 and 5</t>
   </si>
@@ -174,9 +174,6 @@
   </si>
   <si>
     <t>-41.11</t>
-  </si>
-  <si>
-    <t>4749.57</t>
   </si>
   <si>
     <t>AC</t>
@@ -557,7 +554,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="37" x14ac:knownFonts="1">
+  <fonts count="36" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -681,12 +678,6 @@
     </font>
     <font>
       <b/>
-      <sz val="20"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="14"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1599,10 +1590,10 @@
     <xf numFmtId="2" fontId="0" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1611,13 +1602,13 @@
     <xf numFmtId="164" fontId="19" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1626,13 +1617,13 @@
     <xf numFmtId="2" fontId="0" fillId="3" borderId="35" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1641,13 +1632,13 @@
     <xf numFmtId="2" fontId="0" fillId="3" borderId="39" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1656,26 +1647,26 @@
     <xf numFmtId="2" fontId="0" fillId="3" borderId="43" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="47" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="36" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1684,15 +1675,21 @@
     <xf numFmtId="2" fontId="0" fillId="3" borderId="51" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="35" fillId="2" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="51" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1710,25 +1707,19 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="36" fillId="2" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="51" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2057,29 +2048,29 @@
     </row>
     <row r="2" spans="2:13" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="1"/>
-      <c r="C2" s="60" t="s">
+      <c r="C2" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="61"/>
+      <c r="D2" s="65"/>
       <c r="E2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="60" t="s">
+      <c r="F2" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="61"/>
-      <c r="H2" s="60" t="s">
+      <c r="G2" s="65"/>
+      <c r="H2" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="61"/>
-      <c r="J2" s="60" t="s">
+      <c r="I2" s="65"/>
+      <c r="J2" s="64" t="s">
         <v>5</v>
       </c>
-      <c r="K2" s="61"/>
-      <c r="L2" s="60" t="s">
+      <c r="K2" s="65"/>
+      <c r="L2" s="64" t="s">
         <v>6</v>
       </c>
-      <c r="M2" s="61"/>
+      <c r="M2" s="65"/>
     </row>
     <row r="3" spans="2:13" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="3"/>
@@ -2293,8 +2284,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="69" t="s">
-        <v>130</v>
+      <c r="B1" s="71" t="s">
+        <v>129</v>
       </c>
       <c r="C1" s="63"/>
       <c r="D1" s="63"/>
@@ -2302,15 +2293,15 @@
     <row r="2" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="19"/>
       <c r="C2" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" s="20" t="s">
         <v>122</v>
-      </c>
-      <c r="D2" s="20" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="21" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C3" s="22">
         <v>2.3235041965896191E-2</v>
@@ -2321,7 +2312,7 @@
     </row>
     <row r="4" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="21" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C4" s="22">
         <v>-2.4010626649669641E-2</v>
@@ -2332,7 +2323,7 @@
     </row>
     <row r="5" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="21" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C5" s="22">
         <v>3.061374543613862E-2</v>
@@ -2343,7 +2334,7 @@
     </row>
     <row r="6" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C6" s="22">
         <v>0.22181641642497621</v>
@@ -2354,7 +2345,7 @@
     </row>
     <row r="7" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="21" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C7" s="22">
         <v>0.23164532616789241</v>
@@ -2365,7 +2356,7 @@
     </row>
     <row r="8" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="21" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C8" s="22">
         <v>-0.1056222474011311</v>
@@ -2376,7 +2367,7 @@
     </row>
     <row r="9" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="21" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C9" s="22">
         <v>0.15234345741177441</v>
@@ -2387,7 +2378,7 @@
     </row>
     <row r="10" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C10" s="22">
         <v>3.5123575115592477E-2</v>
@@ -2398,7 +2389,7 @@
     </row>
     <row r="11" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="21" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C11" s="22">
         <v>-9.8811963996663532E-2</v>
@@ -2409,7 +2400,7 @@
     </row>
     <row r="12" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="21" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C12" s="22">
         <v>0.25407444787154981</v>
@@ -2436,17 +2427,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="70" t="s">
-        <v>135</v>
+      <c r="B1" s="62" t="s">
+        <v>134</v>
       </c>
       <c r="C1" s="63"/>
     </row>
     <row r="2" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="31" t="s">
+        <v>135</v>
+      </c>
+      <c r="C2" s="32" t="s">
         <v>136</v>
-      </c>
-      <c r="C2" s="32" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="3" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2459,7 +2450,7 @@
     </row>
     <row r="4" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="34" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C4" s="33">
         <v>31</v>
@@ -2549,8 +2540,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="71" t="s">
-        <v>139</v>
+      <c r="B1" s="72" t="s">
+        <v>138</v>
       </c>
       <c r="C1" s="63"/>
       <c r="D1" s="63"/>
@@ -2565,31 +2556,31 @@
     <row r="2" spans="2:11" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="40"/>
       <c r="C2" s="41" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2" s="41" t="s">
         <v>140</v>
       </c>
-      <c r="D2" s="41" t="s">
+      <c r="E2" s="41" t="s">
         <v>141</v>
       </c>
-      <c r="E2" s="41" t="s">
+      <c r="F2" s="41" t="s">
         <v>142</v>
       </c>
-      <c r="F2" s="41" t="s">
+      <c r="G2" s="41" t="s">
         <v>143</v>
       </c>
-      <c r="G2" s="41" t="s">
+      <c r="H2" s="41" t="s">
         <v>144</v>
       </c>
-      <c r="H2" s="41" t="s">
+      <c r="I2" s="41" t="s">
         <v>145</v>
       </c>
-      <c r="I2" s="41" t="s">
+      <c r="J2" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="J2" s="41" t="s">
+      <c r="K2" s="41" t="s">
         <v>147</v>
-      </c>
-      <c r="K2" s="41" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="3" spans="2:11" ht="25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2597,7 +2588,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="43" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D3" s="43">
         <v>4</v>
@@ -2629,7 +2620,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D4" s="43">
         <v>4</v>
@@ -2661,7 +2652,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D5" s="43">
         <v>3</v>
@@ -2693,7 +2684,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D6" s="43">
         <v>3</v>
@@ -2739,8 +2730,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:5" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="72" t="s">
-        <v>151</v>
+      <c r="B1" s="73" t="s">
+        <v>150</v>
       </c>
       <c r="C1" s="63"/>
       <c r="D1" s="63"/>
@@ -2749,13 +2740,13 @@
     <row r="2" spans="2:5" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="35"/>
       <c r="C2" s="36" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D2" s="36" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E2" s="36" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="2:5" ht="25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2763,10 +2754,10 @@
         <v>0</v>
       </c>
       <c r="C3" s="38" t="s">
+        <v>152</v>
+      </c>
+      <c r="D3" s="38" t="s">
         <v>153</v>
-      </c>
-      <c r="D3" s="38" t="s">
-        <v>154</v>
       </c>
       <c r="E3" s="39">
         <v>0.19077767395010881</v>
@@ -2777,10 +2768,10 @@
         <v>1</v>
       </c>
       <c r="C4" s="38" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D4" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E4" s="39">
         <v>0.19122240005791241</v>
@@ -2791,10 +2782,10 @@
         <v>2</v>
       </c>
       <c r="C5" s="38" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E5" s="39">
         <v>0.81587740225031424</v>
@@ -2805,10 +2796,10 @@
         <v>3</v>
       </c>
       <c r="C6" s="38" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E6" s="39">
         <v>0.73960175688119334</v>
@@ -2833,8 +2824,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:5" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="73" t="s">
-        <v>157</v>
+      <c r="B1" s="74" t="s">
+        <v>156</v>
       </c>
       <c r="C1" s="63"/>
       <c r="D1" s="63"/>
@@ -2843,13 +2834,13 @@
     <row r="2" spans="2:5" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="45"/>
       <c r="C2" s="46" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D2" s="46" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E2" s="46" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="2:5" ht="25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2857,10 +2848,10 @@
         <v>0</v>
       </c>
       <c r="C3" s="48" t="s">
+        <v>152</v>
+      </c>
+      <c r="D3" s="48" t="s">
         <v>153</v>
-      </c>
-      <c r="D3" s="48" t="s">
-        <v>154</v>
       </c>
       <c r="E3" s="49">
         <v>0.3707348443913232</v>
@@ -2871,10 +2862,10 @@
         <v>1</v>
       </c>
       <c r="C4" s="48" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D4" s="48" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E4" s="49">
         <v>0.34070541055434389</v>
@@ -2885,10 +2876,10 @@
         <v>2</v>
       </c>
       <c r="C5" s="48" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D5" s="48" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E5" s="49">
         <v>0.33356490637033559</v>
@@ -2899,10 +2890,10 @@
         <v>3</v>
       </c>
       <c r="C6" s="48" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D6" s="48" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E6" s="49">
         <v>0.31002531717376391</v>
@@ -2928,8 +2919,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="73" t="s">
-        <v>158</v>
+      <c r="B1" s="74" t="s">
+        <v>157</v>
       </c>
       <c r="C1" s="63"/>
       <c r="D1" s="63"/>
@@ -2944,31 +2935,31 @@
     <row r="2" spans="2:11" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="45"/>
       <c r="C2" s="46" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2" s="46" t="s">
         <v>140</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="E2" s="46" t="s">
         <v>141</v>
       </c>
-      <c r="E2" s="46" t="s">
+      <c r="F2" s="46" t="s">
         <v>142</v>
       </c>
-      <c r="F2" s="46" t="s">
+      <c r="G2" s="46" t="s">
         <v>143</v>
       </c>
-      <c r="G2" s="46" t="s">
+      <c r="H2" s="46" t="s">
         <v>144</v>
       </c>
-      <c r="H2" s="46" t="s">
+      <c r="I2" s="46" t="s">
         <v>145</v>
       </c>
-      <c r="I2" s="46" t="s">
+      <c r="J2" s="46" t="s">
         <v>146</v>
       </c>
-      <c r="J2" s="46" t="s">
+      <c r="K2" s="46" t="s">
         <v>147</v>
-      </c>
-      <c r="K2" s="46" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="3" spans="2:11" ht="25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2976,7 +2967,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="48" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D3" s="48">
         <v>4</v>
@@ -3008,7 +2999,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="48" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D4" s="48">
         <v>4</v>
@@ -3040,7 +3031,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="48" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D5" s="48">
         <v>3</v>
@@ -3072,7 +3063,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="48" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D6" s="48">
         <v>3</v>
@@ -3117,8 +3108,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="74" t="s">
-        <v>159</v>
+      <c r="B1" s="75" t="s">
+        <v>158</v>
       </c>
       <c r="C1" s="63"/>
       <c r="D1" s="63"/>
@@ -3126,15 +3117,15 @@
     <row r="2" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="50"/>
       <c r="C2" s="51" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D2" s="51" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="52" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C3" s="53">
         <v>3160</v>
@@ -3156,7 +3147,7 @@
     </row>
     <row r="5" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="52" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C5" s="53">
         <v>3100.5364682198879</v>
@@ -3167,7 +3158,7 @@
     </row>
     <row r="6" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="52" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C6" s="53">
         <v>-142779.98000000001</v>
@@ -3178,7 +3169,7 @@
     </row>
     <row r="7" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="52" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C7" s="53">
         <v>-181.77</v>
@@ -3189,7 +3180,7 @@
     </row>
     <row r="8" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="52" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C8" s="53">
         <v>-67.454999999999998</v>
@@ -3200,7 +3191,7 @@
     </row>
     <row r="9" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="52" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C9" s="53">
         <v>-31.987500000000001</v>
@@ -3211,7 +3202,7 @@
     </row>
     <row r="10" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="52" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C10" s="53">
         <v>-0.02</v>
@@ -3388,19 +3379,19 @@
       <c r="B3" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="6" t="s">
         <v>36</v>
       </c>
     </row>
@@ -3408,180 +3399,180 @@
       <c r="B4" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="G4" s="9" t="s">
-        <v>42</v>
+      <c r="G4" s="76">
+        <v>4749.57</v>
       </c>
     </row>
     <row r="5" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="D5" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="E5" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="F5" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="G5" s="6" t="s">
         <v>47</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="D6" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="E6" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="F6" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="G6" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="D7" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="E7" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="F7" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="G7" s="6" t="s">
         <v>59</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="D8" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="F8" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="G8" s="6" t="s">
         <v>63</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="9" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="D9" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D9" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="6" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="D10" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="E10" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="F10" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="G10" s="6" t="s">
         <v>72</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="11" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="6" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="D12" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="E12" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="F12" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="G12" s="6" t="s">
         <v>80</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -3603,8 +3594,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="64" t="s">
-        <v>82</v>
+      <c r="B1" s="66" t="s">
+        <v>81</v>
       </c>
       <c r="C1" s="63"/>
       <c r="D1" s="63"/>
@@ -3624,34 +3615,34 @@
         <v>28</v>
       </c>
       <c r="D2" s="56" t="s">
+        <v>82</v>
+      </c>
+      <c r="E2" s="56" t="s">
         <v>83</v>
       </c>
-      <c r="E2" s="56" t="s">
+      <c r="F2" s="56" t="s">
         <v>84</v>
       </c>
-      <c r="F2" s="56" t="s">
+      <c r="G2" s="56" t="s">
         <v>85</v>
       </c>
-      <c r="G2" s="56" t="s">
+      <c r="H2" s="60" t="s">
         <v>86</v>
       </c>
-      <c r="H2" s="75" t="s">
+      <c r="I2" s="56" t="s">
         <v>87</v>
-      </c>
-      <c r="I2" s="56" t="s">
-        <v>88</v>
       </c>
       <c r="J2" s="56" t="s">
         <v>17</v>
       </c>
       <c r="K2" s="56" t="s">
+        <v>88</v>
+      </c>
+      <c r="L2" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="L2" s="56" t="s">
+      <c r="M2" s="56" t="s">
         <v>90</v>
-      </c>
-      <c r="M2" s="56" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="3" spans="2:13" ht="25" customHeight="1" x14ac:dyDescent="0.2">
@@ -3659,13 +3650,13 @@
         <v>28727</v>
       </c>
       <c r="C3" s="58" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D3" s="58">
         <v>5324</v>
       </c>
       <c r="E3" s="58" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F3" s="58" t="s">
         <v>4</v>
@@ -3673,7 +3664,7 @@
       <c r="G3" s="59">
         <v>74.91</v>
       </c>
-      <c r="H3" s="76">
+      <c r="H3" s="61">
         <v>44354</v>
       </c>
       <c r="I3" s="58">
@@ -3697,13 +3688,13 @@
         <v>53577</v>
       </c>
       <c r="C4" s="58" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D4" s="58">
         <v>9866</v>
       </c>
       <c r="E4" s="58" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F4" s="58" t="s">
         <v>4</v>
@@ -3711,7 +3702,7 @@
       <c r="G4" s="59">
         <v>79.62</v>
       </c>
-      <c r="H4" s="76">
+      <c r="H4" s="61">
         <v>44729</v>
       </c>
       <c r="I4" s="58">
@@ -3735,13 +3726,13 @@
         <v>36992</v>
       </c>
       <c r="C5" s="58" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D5" s="58">
         <v>6521</v>
       </c>
       <c r="E5" s="58" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F5" s="58" t="s">
         <v>4</v>
@@ -3749,7 +3740,7 @@
       <c r="G5" s="59">
         <v>55.55</v>
       </c>
-      <c r="H5" s="76">
+      <c r="H5" s="61">
         <v>44460</v>
       </c>
       <c r="I5" s="58">
@@ -3773,21 +3764,21 @@
         <v>33942</v>
       </c>
       <c r="C6" s="58" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D6" s="58">
         <v>6040</v>
       </c>
       <c r="E6" s="58" t="s">
+        <v>98</v>
+      </c>
+      <c r="F6" s="58" t="s">
         <v>99</v>
-      </c>
-      <c r="F6" s="58" t="s">
-        <v>100</v>
       </c>
       <c r="G6" s="59">
         <v>475.62</v>
       </c>
-      <c r="H6" s="76">
+      <c r="H6" s="61">
         <v>44417</v>
       </c>
       <c r="I6" s="58">
@@ -3811,21 +3802,21 @@
         <v>53920</v>
       </c>
       <c r="C7" s="58" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D7" s="58">
         <v>9940</v>
       </c>
       <c r="E7" s="58" t="s">
+        <v>101</v>
+      </c>
+      <c r="F7" s="58" t="s">
         <v>102</v>
-      </c>
-      <c r="F7" s="58" t="s">
-        <v>103</v>
       </c>
       <c r="G7" s="59">
         <v>395.67</v>
       </c>
-      <c r="H7" s="76">
+      <c r="H7" s="61">
         <v>44740</v>
       </c>
       <c r="I7" s="58">
@@ -3862,18 +3853,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="65"/>
+      <c r="B1" s="67"/>
       <c r="C1" s="63"/>
     </row>
     <row r="2" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="11"/>
       <c r="C2" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C3" s="14">
         <v>355</v>
@@ -3881,7 +3872,7 @@
     </row>
     <row r="4" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C4" s="14">
         <v>13947</v>
@@ -3889,7 +3880,7 @@
     </row>
     <row r="5" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C5" s="14">
         <v>4</v>
@@ -3897,7 +3888,7 @@
     </row>
     <row r="6" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C6" s="14">
         <v>20</v>
@@ -3920,29 +3911,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="65"/>
+      <c r="B1" s="67"/>
       <c r="C1" s="63"/>
     </row>
     <row r="2" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="11"/>
       <c r="C2" s="12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C3" s="14" t="s">
         <v>108</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="4" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" s="14" t="s">
         <v>110</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -3962,20 +3953,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="66" t="s">
-        <v>112</v>
+      <c r="B1" s="68" t="s">
+        <v>111</v>
       </c>
       <c r="C1" s="63"/>
     </row>
     <row r="2" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="15"/>
       <c r="C2" s="16" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="17" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C3" s="18">
         <v>0.42523101515745299</v>
@@ -3983,7 +3974,7 @@
     </row>
     <row r="4" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="17" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C4" s="18">
         <v>4.7242171840913831E-2</v>
@@ -3991,7 +3982,7 @@
     </row>
     <row r="5" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="17" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C5" s="18">
         <v>2.3894794390017829E-11</v>
@@ -4014,20 +4005,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="67" t="s">
-        <v>117</v>
+      <c r="B1" s="69" t="s">
+        <v>116</v>
       </c>
       <c r="C1" s="63"/>
     </row>
     <row r="2" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="27"/>
       <c r="C2" s="28" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="29" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C3" s="30">
         <v>2.8530607940061539E-2</v>
@@ -4035,7 +4026,7 @@
     </row>
     <row r="4" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="29" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C4" s="30">
         <v>6.1547009268820004E-5</v>
@@ -4043,7 +4034,7 @@
     </row>
     <row r="5" spans="2:3" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="29" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C5" s="30">
         <v>1.7467156215665861E-8</v>
@@ -4067,8 +4058,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="68" t="s">
-        <v>121</v>
+      <c r="B1" s="70" t="s">
+        <v>120</v>
       </c>
       <c r="C1" s="63"/>
       <c r="D1" s="63"/>
@@ -4076,15 +4067,15 @@
     <row r="2" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="23"/>
       <c r="C2" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" s="24" t="s">
         <v>122</v>
-      </c>
-      <c r="D2" s="24" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="25" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C3" s="26">
         <v>4.0079423901679158E-2</v>
@@ -4095,7 +4086,7 @@
     </row>
     <row r="4" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="25" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C4" s="26">
         <v>-0.68261251647126298</v>
@@ -4106,7 +4097,7 @@
     </row>
     <row r="5" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="25" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C5" s="26">
         <v>-9.8774743092295281E-2</v>
@@ -4117,7 +4108,7 @@
     </row>
     <row r="6" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="25" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C6" s="26">
         <v>-7.525903216987942E-2</v>
@@ -4128,7 +4119,7 @@
     </row>
     <row r="7" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="25" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C7" s="26">
         <v>7.4356806990677579E-2</v>
@@ -4139,7 +4130,7 @@
     </row>
     <row r="8" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="25" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C8" s="26">
         <v>-6.0210329575816478E-2</v>

</xml_diff>